<commit_message>
Fix Excel dashboard: correct number formatting, show all 8 products, fix column widths and chart placement
</commit_message>
<xml_diff>
--- a/task-2-eda-business-intelligence/sales_dashboard_mockup.xlsx
+++ b/task-2-eda-business-intelligence/sales_dashboard_mockup.xlsx
@@ -18,9 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="8">
     <font>
       <name val="Calibri"/>
@@ -30,48 +28,48 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
+      <color rgb="00111111"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="001A1A2E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -80,7 +78,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A2E"/>
+        <fgColor rgb="000D1B2A"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,27 +88,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F9A825"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="005368A6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A35C2D"/>
+        <fgColor rgb="00C06000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002A9D8F"/>
+        <fgColor rgb="001A7A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E63946"/>
+        <fgColor rgb="00C0392B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
+        <fgColor rgb="00455A64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -118,8 +126,13 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B6CA8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -128,40 +141,54 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -171,58 +198,71 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -362,7 +402,7 @@
             <idx val="2"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="A35C2D"/>
+                <a:srgbClr val="C06000"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -405,7 +445,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Top Products by Revenue ($)</a:t>
+              <a:t>Top 8 Products by Revenue</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -455,21 +495,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Revenue ($)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -482,21 +507,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Product</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -538,7 +548,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Monthly Trend'!B2</f>
+              <f>'Monthly Trend'!B3</f>
             </strRef>
           </tx>
           <spPr>
@@ -559,12 +569,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Monthly Trend'!$A$3:$A$17</f>
+              <f>'Monthly Trend'!$A$4:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Monthly Trend'!$B$3:$B$17</f>
+              <f>'Monthly Trend'!$B$4:$B$18</f>
             </numRef>
           </val>
         </ser>
@@ -573,13 +583,13 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Monthly Trend'!E2</f>
+              <f>'Monthly Trend'!E3</f>
             </strRef>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
               <a:solidFill>
-                <a:srgbClr val="2A9D8F"/>
+                <a:srgbClr val="1A7A4A"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -594,12 +604,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Monthly Trend'!$A$3:$A$17</f>
+              <f>'Monthly Trend'!$A$4:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Monthly Trend'!$E$3:$E$17</f>
+              <f>'Monthly Trend'!$E$4:$E$18</f>
             </numRef>
           </val>
         </ser>
@@ -696,28 +706,28 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Monthly Trend'!C2</f>
+              <f>'Monthly Trend'!C3</f>
             </strRef>
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="A35C2D"/>
+              <a:srgbClr val="C06000"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
-                <a:srgbClr val="A35C2D"/>
+                <a:srgbClr val="C06000"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Monthly Trend'!$A$3:$A$17</f>
+              <f>'Monthly Trend'!$A$4:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Monthly Trend'!$C$3:$C$17</f>
+              <f>'Monthly Trend'!$C$4:$C$18</f>
             </numRef>
           </val>
         </ser>
@@ -800,7 +810,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue by Product Category</a:t>
+              <a:t>Revenue by Product Category ($)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -904,110 +914,6 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue per Customer by Age Group</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Category &amp; Segments'!J4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2A9D8F"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="2A9D8F"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Category &amp; Segments'!$G$5:$G$9</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Category &amp; Segments'!$J$5:$J$9</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Revenue/Customer ($)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
               <a:t>Category Revenue Share</a:t>
             </a:r>
           </a:p>
@@ -1056,7 +962,7 @@
             <idx val="2"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="A35C2D"/>
+                <a:srgbClr val="C06000"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -1067,7 +973,7 @@
             <idx val="3"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2A9D8F"/>
+                <a:srgbClr val="1A7A4A"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -1097,16 +1003,224 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Revenue per Customer by Age Group</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Category &amp; Segments'!K4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="5368A6"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="5368A6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Category &amp; Segments'!$H$5:$H$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Category &amp; Segments'!$K$5:$K$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue / Customer ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Total Revenue by Age Group ($)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Category &amp; Segments'!I4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="1A7A4A"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="1A7A4A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Category &amp; Segments'!$H$5:$H$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Category &amp; Segments'!$I$5:$I$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5040000" cy="3600000"/>
+    <ext cx="5040000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1123,12 +1237,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>6</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="4320000"/>
+    <ext cx="7200000" cy="4680000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1152,10 +1266,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9360000" cy="5040000"/>
+    <ext cx="10080000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1174,10 +1288,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>38</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9360000" cy="4320000"/>
+    <ext cx="10080000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1221,12 +1335,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="4320000"/>
+    <ext cx="5040000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1243,12 +1357,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>0</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5040000" cy="3600000"/>
+    <ext cx="6480000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1258,6 +1372,28 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1555,577 +1691,626 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SALES PERFORMANCE EXECUTIVE DASHBOARD</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
+    <row r="2" ht="5" customHeight="1"/>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>TOTAL REVENUE</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>TOTAL ORDERS</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>AVG ORDER VALUE</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>GROSS MARGIN</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>RETURN RATE</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>$5,328,492.40</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>$5,328,492</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>1,250</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>$4,262.79</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>20.32%</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>5.20%</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1"/>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="5" ht="5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr"/>
+      <c r="C5" s="12" t="inlineStr"/>
+      <c r="E5" s="12" t="inlineStr"/>
+      <c r="G5" s="12" t="inlineStr"/>
+      <c r="I5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  TOP PRODUCTS BY REVENUE</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  REVENUE BY SALES CHANNEL</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Product Name</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>Avg Price ($)</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>Return Rate (%)</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>Sales Channel</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Return %</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr">
+      <c r="I8" s="15" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="J8" s="14" t="inlineStr">
-        <is>
-          <t>Profit Margin %</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>Gross Profit ($)</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>Margin %</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Smart Watch</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <v>1368209.84</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="18" t="n">
         <v>152</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <v>6042.26</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.07240000000000001</v>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="H9" s="17" t="n">
         <v>2464279.62</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="18" t="n">
         <v>592</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="17" t="n">
+        <v>488850.64</v>
+      </c>
+      <c r="K9" s="19" t="n">
         <v>0.1984</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Mechanical Keyboard</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="21" t="n">
         <v>899189.76</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="22" t="n">
         <v>156</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="21" t="n">
         <v>3499.89</v>
       </c>
-      <c r="E10" s="22" t="n">
+      <c r="E10" s="23" t="n">
         <v>0.0128</v>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G10" s="20" t="inlineStr">
         <is>
           <t>Mobile App</t>
         </is>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="21" t="n">
         <v>2054498.79</v>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="22" t="n">
         <v>456</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="21" t="n">
+        <v>441586.34</v>
+      </c>
+      <c r="K10" s="23" t="n">
         <v>0.2149</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Webcam Pro</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="17" t="n">
         <v>798137.5</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="18" t="n">
         <v>169</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="17" t="n">
         <v>3170.67</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>0.0473</v>
       </c>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>Retail Store</t>
         </is>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="17" t="n">
         <v>809713.99</v>
       </c>
-      <c r="I11" s="17" t="n">
+      <c r="I11" s="18" t="n">
         <v>202</v>
       </c>
-      <c r="J11" s="18" t="n">
+      <c r="J11" s="17" t="n">
+        <v>152312.33</v>
+      </c>
+      <c r="K11" s="19" t="n">
         <v>0.1881</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+    <row r="12" ht="8" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Bluetooth Headphones</t>
         </is>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="21" t="n">
         <v>655422.34</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="22" t="n">
         <v>151</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="21" t="n">
         <v>2654.19</v>
       </c>
-      <c r="E12" s="22" t="n">
+      <c r="E12" s="23" t="n">
         <v>0.053</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Portable Speaker</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B13" s="17" t="n">
         <v>600264</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="18" t="n">
         <v>157</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="17" t="n">
         <v>2208.11</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <v>0.0764</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MARKETING CAMPAIGN SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>USB-C Hub</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n">
+      <c r="B14" s="21" t="n">
         <v>506903.56</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="22" t="n">
         <v>161</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="21" t="n">
         <v>1911.33</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="23" t="n">
         <v>0.0683</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>Revenue ($)</t>
+        </is>
+      </c>
+      <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="inlineStr">
+        <is>
+          <t>Gross Profit ($)</t>
+        </is>
+      </c>
+      <c r="K14" s="15" t="inlineStr">
+        <is>
+          <t>Margin %</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Laptop Stand</t>
         </is>
       </c>
-      <c r="B15" s="16" t="n">
+      <c r="B15" s="17" t="n">
         <v>296637.2</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="18" t="n">
         <v>143</v>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="17" t="n">
         <v>1307.75</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="19" t="n">
         <v>0.049</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Search Ads</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>1034918.19</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>219</v>
+      </c>
+      <c r="J15" s="17" t="n">
+        <v>276020.3</v>
+      </c>
+      <c r="K15" s="19" t="n">
+        <v>0.2667</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Wireless Mouse</t>
         </is>
       </c>
-      <c r="B16" s="20" t="n">
+      <c r="B16" s="21" t="n">
         <v>203728.2</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="22" t="n">
         <v>161</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="21" t="n">
         <v>798.97</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="23" t="n">
         <v>0.0373</v>
       </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="H16" s="21" t="n">
+        <v>946146.16</v>
+      </c>
+      <c r="I16" s="22" t="n">
+        <v>217</v>
+      </c>
+      <c r="J16" s="21" t="n">
+        <v>198461.91</v>
+      </c>
+      <c r="K16" s="23" t="n">
+        <v>0.2098</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Referral</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>904176.23</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>205</v>
+      </c>
+      <c r="J17" s="17" t="n">
+        <v>185194.66</v>
+      </c>
+      <c r="K17" s="19" t="n">
+        <v>0.2048</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  PERFORMANCE BY REGION</t>
         </is>
       </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MARKETING CAMPAIGN SUMMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>Email Offer</t>
+        </is>
+      </c>
+      <c r="H18" s="21" t="n">
+        <v>844455.76</v>
+      </c>
+      <c r="I18" s="22" t="n">
+        <v>222</v>
+      </c>
+      <c r="J18" s="21" t="n">
+        <v>117325.28</v>
+      </c>
+      <c r="K18" s="23" t="n">
+        <v>0.1389</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>Gross Profit ($)</t>
         </is>
       </c>
-      <c r="E21" s="23" t="inlineStr">
-        <is>
-          <t>Return Rate (%)</t>
-        </is>
-      </c>
-      <c r="G21" s="24" t="inlineStr">
-        <is>
-          <t>Campaign</t>
-        </is>
-      </c>
-      <c r="H21" s="24" t="inlineStr">
-        <is>
-          <t>Revenue ($)</t>
-        </is>
-      </c>
-      <c r="I21" s="24" t="inlineStr">
-        <is>
-          <t>Orders</t>
-        </is>
-      </c>
-      <c r="J21" s="24" t="inlineStr">
-        <is>
-          <t>Profit Margin %</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Return %</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="H19" s="17" t="n">
+        <v>809556.17</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>191</v>
+      </c>
+      <c r="J19" s="17" t="n">
+        <v>158623.78</v>
+      </c>
+      <c r="K19" s="19" t="n">
+        <v>0.1959</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n">
+      <c r="B20" s="17" t="n">
         <v>1451298.87</v>
       </c>
-      <c r="C22" s="17" t="n">
+      <c r="C20" s="18" t="n">
         <v>339</v>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D20" s="17" t="n">
         <v>273233.41</v>
       </c>
-      <c r="E22" s="18" t="n">
+      <c r="E20" s="19" t="n">
         <v>0.0383</v>
       </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>Search Ads</t>
-        </is>
-      </c>
-      <c r="H22" s="16" t="n">
-        <v>1034918.19</v>
-      </c>
-      <c r="I22" s="17" t="n">
-        <v>219</v>
-      </c>
-      <c r="J22" s="18" t="n">
-        <v>0.2667</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>Festive Sale</t>
+        </is>
+      </c>
+      <c r="H20" s="21" t="n">
+        <v>789239.89</v>
+      </c>
+      <c r="I20" s="22" t="n">
+        <v>196</v>
+      </c>
+      <c r="J20" s="21" t="n">
+        <v>147123.38</v>
+      </c>
+      <c r="K20" s="23" t="n">
+        <v>0.1864</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B21" s="21" t="n">
         <v>1301485.12</v>
       </c>
-      <c r="C23" s="21" t="n">
+      <c r="C21" s="22" t="n">
         <v>320</v>
       </c>
-      <c r="D23" s="20" t="n">
+      <c r="D21" s="21" t="n">
         <v>250426.93</v>
       </c>
-      <c r="E23" s="22" t="n">
+      <c r="E21" s="23" t="n">
         <v>0.07190000000000001</v>
       </c>
-      <c r="G23" s="19" t="inlineStr">
-        <is>
-          <t>Organic</t>
-        </is>
-      </c>
-      <c r="H23" s="20" t="n">
-        <v>946146.16</v>
-      </c>
-      <c r="I23" s="21" t="n">
-        <v>217</v>
-      </c>
-      <c r="J23" s="22" t="n">
-        <v>0.2098</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B22" s="17" t="n">
         <v>1288064.81</v>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C22" s="18" t="n">
         <v>299</v>
       </c>
-      <c r="D24" s="16" t="n">
+      <c r="D22" s="17" t="n">
         <v>315503.55</v>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="E22" s="19" t="n">
         <v>0.0569</v>
       </c>
-      <c r="G24" s="15" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="H24" s="16" t="n">
-        <v>904176.23</v>
-      </c>
-      <c r="I24" s="17" t="n">
-        <v>205</v>
-      </c>
-      <c r="J24" s="18" t="n">
-        <v>0.2048</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n">
+      <c r="B23" s="21" t="n">
         <v>1287643.6</v>
       </c>
-      <c r="C25" s="21" t="n">
+      <c r="C23" s="22" t="n">
         <v>292</v>
       </c>
-      <c r="D25" s="20" t="n">
+      <c r="D23" s="21" t="n">
         <v>243585.42</v>
       </c>
-      <c r="E25" s="22" t="n">
+      <c r="E23" s="23" t="n">
         <v>0.0411</v>
       </c>
-      <c r="G25" s="19" t="inlineStr">
-        <is>
-          <t>Email Offer</t>
-        </is>
-      </c>
-      <c r="H25" s="20" t="n">
-        <v>844455.76</v>
-      </c>
-      <c r="I25" s="21" t="n">
-        <v>222</v>
-      </c>
-      <c r="J25" s="22" t="n">
-        <v>0.1389</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="G26" s="15" t="inlineStr">
-        <is>
-          <t>Influencer</t>
-        </is>
-      </c>
-      <c r="H26" s="16" t="n">
-        <v>809556.17</v>
-      </c>
-      <c r="I26" s="17" t="n">
-        <v>191</v>
-      </c>
-      <c r="J26" s="18" t="n">
-        <v>0.1959</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="G27" s="19" t="inlineStr">
-        <is>
-          <t>Festive Sale</t>
-        </is>
-      </c>
-      <c r="H27" s="20" t="n">
-        <v>789239.89</v>
-      </c>
-      <c r="I27" s="21" t="n">
-        <v>196</v>
-      </c>
-      <c r="J27" s="22" t="n">
-        <v>0.1864</v>
-      </c>
-    </row>
+    </row>
+    <row r="24" ht="8" customHeight="1"/>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="B3:C3"/>
+  <mergeCells count="20">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G7:K7"/>
     <mergeCell ref="A7:E7"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G7:J7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2138,408 +2323,410 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>MONTHLY SALES AND PROFIT TREND</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+    <row r="2" ht="5" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Order Month</t>
         </is>
       </c>
-      <c r="B2" s="24" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>Total Revenue ($)</t>
         </is>
       </c>
-      <c r="C2" s="24" t="inlineStr">
-        <is>
-          <t>Order Count</t>
-        </is>
-      </c>
-      <c r="D2" s="24" t="inlineStr">
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
         <is>
           <t>Total Cost ($)</t>
         </is>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E3" s="27" t="inlineStr">
         <is>
           <t>Gross Profit ($)</t>
         </is>
       </c>
-      <c r="F2" s="24" t="inlineStr">
+      <c r="F3" s="27" t="inlineStr">
         <is>
           <t>Profit Margin %</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>414508.3</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C4" s="18" t="n">
         <v>101</v>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D4" s="17" t="n">
         <v>336284.42</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E4" s="17" t="n">
         <v>78223.88</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>0.1887</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>2025-02</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B5" s="21" t="n">
         <v>381797.56</v>
       </c>
-      <c r="C4" s="21" t="n">
+      <c r="C5" s="22" t="n">
         <v>84</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D5" s="21" t="n">
         <v>282834.36</v>
       </c>
-      <c r="E4" s="20" t="n">
+      <c r="E5" s="21" t="n">
         <v>98963.2</v>
       </c>
-      <c r="F4" s="22" t="n">
+      <c r="F5" s="23" t="n">
         <v>0.2592</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>2025-03</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>253183.26</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C6" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D6" s="17" t="n">
         <v>204061.76</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E6" s="17" t="n">
         <v>49121.5</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.194</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
+      <c r="B7" s="21" t="n">
         <v>361993.81</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C7" s="22" t="n">
         <v>88</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D7" s="21" t="n">
         <v>299647.47</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E7" s="21" t="n">
         <v>62346.34</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F7" s="23" t="n">
         <v>0.1722</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B8" s="17" t="n">
         <v>332373.01</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C8" s="18" t="n">
         <v>86</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <v>270547.12</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E8" s="17" t="n">
         <v>61825.89</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>0.186</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B9" s="21" t="n">
         <v>373196.49</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C9" s="22" t="n">
         <v>77</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D9" s="21" t="n">
         <v>305755.34</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E9" s="21" t="n">
         <v>67441.14999999999</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F9" s="23" t="n">
         <v>0.1807</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B10" s="17" t="n">
         <v>397458.33</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C10" s="18" t="n">
         <v>88</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D10" s="17" t="n">
         <v>318768.7</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E10" s="17" t="n">
         <v>78689.63</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.198</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>2025-08</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B11" s="21" t="n">
         <v>334842.66</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C11" s="22" t="n">
         <v>94</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D11" s="21" t="n">
         <v>275722.86</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E11" s="21" t="n">
         <v>59119.8</v>
       </c>
-      <c r="F10" s="22" t="n">
+      <c r="F11" s="23" t="n">
         <v>0.1766</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B12" s="17" t="n">
         <v>345674.85</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C12" s="18" t="n">
         <v>77</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D12" s="17" t="n">
         <v>279138.65</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E12" s="17" t="n">
         <v>66536.2</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F12" s="19" t="n">
         <v>0.1925</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B13" s="21" t="n">
         <v>364085.7</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C13" s="22" t="n">
         <v>77</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D13" s="21" t="n">
         <v>292943.39</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E13" s="21" t="n">
         <v>71142.31</v>
       </c>
-      <c r="F12" s="22" t="n">
+      <c r="F13" s="23" t="n">
         <v>0.1954</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>2025-11</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B14" s="17" t="n">
         <v>330265.79</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C14" s="18" t="n">
         <v>84</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D14" s="17" t="n">
         <v>264816.02</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E14" s="17" t="n">
         <v>65449.77</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F14" s="19" t="n">
         <v>0.1982</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n">
+      <c r="B15" s="21" t="n">
         <v>326024.85</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C15" s="22" t="n">
         <v>87</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D15" s="21" t="n">
         <v>264659.61</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E15" s="21" t="n">
         <v>61365.24</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F15" s="23" t="n">
         <v>0.1882</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="B15" s="16" t="n">
+      <c r="B16" s="17" t="n">
         <v>441892.25</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <v>89</v>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D16" s="17" t="n">
         <v>307375.01</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E16" s="17" t="n">
         <v>134517.24</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F16" s="19" t="n">
         <v>0.3044</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="B16" s="20" t="n">
+      <c r="B17" s="21" t="n">
         <v>388410.22</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C17" s="22" t="n">
         <v>74</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D17" s="21" t="n">
         <v>317467.41</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E17" s="21" t="n">
         <v>70942.81</v>
       </c>
-      <c r="F16" s="22" t="n">
+      <c r="F17" s="23" t="n">
         <v>0.1826</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="28" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n">
+      <c r="B18" s="17" t="n">
         <v>282785.32</v>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C18" s="18" t="n">
         <v>64</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D18" s="17" t="n">
         <v>225720.97</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E18" s="17" t="n">
         <v>57064.35</v>
       </c>
-      <c r="F17" s="18" t="n">
+      <c r="F18" s="19" t="n">
         <v>0.2018</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="n">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="n">
         <v>5328492.4</v>
       </c>
-      <c r="C18" s="28" t="n">
+      <c r="C19" s="32" t="n">
         <v>1250</v>
       </c>
-      <c r="D18" s="27" t="n">
+      <c r="D19" s="31" t="n">
         <v>4245778.09</v>
       </c>
-      <c r="E18" s="27" t="n">
+      <c r="E19" s="31" t="n">
         <v>1082548.82</v>
       </c>
-      <c r="F18" s="29" t="n">
+      <c r="F19" s="33" t="n">
         <v>0.2032</v>
       </c>
     </row>
+    <row r="20" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -2555,257 +2742,260 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>CATEGORY &amp; SEGMENT BREAKDOWNS</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="2" ht="5" customHeight="1"/>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  SALES BY PRODUCT CATEGORY</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">  SALES BY CUSTOMER SEGMENT</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Avg Price ($)</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Gross Profit ($)</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>Profit Margin %</t>
-        </is>
-      </c>
-      <c r="G4" s="24" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Margin %</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>Age Group</t>
         </is>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="I4" s="24" t="inlineStr">
+      <c r="J4" s="15" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="J4" s="24" t="inlineStr">
-        <is>
-          <t>Revenue/Customer ($)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>Rev/Customer ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Accessories</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>1609821.52</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="18" t="n">
         <v>478</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="17" t="n">
         <v>2055.11</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="17" t="n">
         <v>345746.17</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>0.2148</v>
       </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="H5" s="28" t="inlineStr">
         <is>
           <t>18-24</t>
         </is>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="I5" s="17" t="n">
         <v>884965.42</v>
       </c>
-      <c r="I5" s="17" t="n">
+      <c r="J5" s="18" t="n">
         <v>210</v>
       </c>
-      <c r="J5" s="16" t="n">
+      <c r="K5" s="17" t="n">
         <v>5746.53</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Wearables</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
+      <c r="B6" s="21" t="n">
         <v>1368209.84</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="22" t="n">
         <v>152</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="21" t="n">
         <v>6042.26</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="21" t="n">
         <v>208448.69</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="23" t="n">
         <v>0.1524</v>
       </c>
-      <c r="G6" s="19" t="inlineStr">
+      <c r="H6" s="29" t="inlineStr">
         <is>
           <t>25-34</t>
         </is>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="I6" s="21" t="n">
         <v>1032052.93</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="J6" s="22" t="n">
         <v>246</v>
       </c>
-      <c r="J6" s="20" t="n">
+      <c r="K6" s="21" t="n">
         <v>5639.63</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Audio</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="17" t="n">
         <v>1255686.34</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="18" t="n">
         <v>308</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="17" t="n">
         <v>2426.8</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="17" t="n">
         <v>264390.68</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.2106</v>
       </c>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="H7" s="28" t="inlineStr">
         <is>
           <t>35-44</t>
         </is>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="I7" s="17" t="n">
         <v>1206867.84</v>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="J7" s="18" t="n">
         <v>268</v>
       </c>
-      <c r="J7" s="16" t="n">
+      <c r="K7" s="17" t="n">
         <v>6004.32</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="21" t="n">
         <v>1094774.7</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="22" t="n">
         <v>312</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="21" t="n">
         <v>2316.83</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="21" t="n">
         <v>264163.77</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="23" t="n">
         <v>0.2413</v>
       </c>
-      <c r="G8" s="19" t="inlineStr">
+      <c r="H8" s="29" t="inlineStr">
         <is>
           <t>45-54</t>
         </is>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="I8" s="21" t="n">
         <v>1059588.09</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="J8" s="22" t="n">
         <v>267</v>
       </c>
-      <c r="J8" s="20" t="n">
+      <c r="K8" s="21" t="n">
         <v>5271.58</v>
       </c>
     </row>
-    <row r="9">
-      <c r="G9" s="15" t="inlineStr">
+    <row r="9" ht="15" customHeight="1">
+      <c r="H9" s="28" t="inlineStr">
         <is>
           <t>55+</t>
         </is>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="I9" s="17" t="n">
         <v>1145018.12</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="J9" s="18" t="n">
         <v>259</v>
       </c>
-      <c r="J9" s="16" t="n">
+      <c r="K9" s="17" t="n">
         <v>6222.92</v>
       </c>
     </row>
+    <row r="10" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="H3:K3"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Rebuild Excel: professional format, conditional colours, freeze panes, correct US number format
</commit_message>
<xml_diff>
--- a/task-2-eda-business-intelligence/sales_dashboard_mockup.xlsx
+++ b/task-2-eda-business-intelligence/sales_dashboard_mockup.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,7 +31,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -43,7 +43,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="17"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -66,10 +66,16 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -123,12 +129,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B6CA8"/>
+        <fgColor rgb="00E8F8F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B4F72"/>
       </patternFill>
     </fill>
   </fills>
@@ -142,31 +163,37 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </left>
       <right style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </right>
       <top style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </bottom>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00BBBBBB"/>
       </right>
-      <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00888888"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -187,82 +214,97 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -343,7 +385,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -434,7 +476,7 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -445,7 +487,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Top 8 Products by Revenue</a:t>
+              <a:t>Top 8 Products — Revenue ($)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -523,7 +565,7 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -552,7 +594,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="5368A6"/>
               </a:solidFill>
@@ -587,7 +629,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="1A7A4A"/>
               </a:solidFill>
@@ -680,7 +722,7 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -799,7 +841,7 @@
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -810,7 +852,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue by Product Category ($)</a:t>
+              <a:t>Revenue by Category ($)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -872,21 +914,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Revenue ($)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -903,7 +930,7 @@
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -1005,7 +1032,7 @@
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -1016,7 +1043,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue per Customer by Age Group</a:t>
+              <a:t>Revenue per Customer by Age ($)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1078,21 +1105,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Revenue / Customer ($)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1109,7 +1121,7 @@
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="26"/>
   <chart>
     <title>
       <tx>
@@ -1182,21 +1194,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Revenue ($)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1242,7 +1239,7 @@
       <row>24</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="4680000"/>
+    <ext cx="7200000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1688,26 +1685,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002F6F73"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="2" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SALES PERFORMANCE EXECUTIVE DASHBOARD</t>
@@ -1742,7 +1740,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>$5,328,492</t>
@@ -1769,7 +1767,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="5" customHeight="1">
+    <row r="5" ht="4" customHeight="1">
       <c r="A5" s="12" t="inlineStr"/>
       <c r="C5" s="12" t="inlineStr"/>
       <c r="E5" s="12" t="inlineStr"/>
@@ -1789,7 +1787,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
+    <row r="8" ht="26" customHeight="1">
       <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Product Name</t>
@@ -1841,7 +1839,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Smart Watch</t>
@@ -1873,47 +1871,47 @@
       <c r="J9" s="17" t="n">
         <v>488850.64</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="20" t="n">
         <v>0.1984</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Mechanical Keyboard</t>
         </is>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="22" t="n">
         <v>899189.76</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>156</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="22" t="n">
         <v>3499.89</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="24" t="n">
         <v>0.0128</v>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Mobile App</t>
         </is>
       </c>
-      <c r="H10" s="21" t="n">
+      <c r="H10" s="22" t="n">
         <v>2054498.79</v>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="I10" s="23" t="n">
         <v>456</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="J10" s="22" t="n">
         <v>441586.34</v>
       </c>
-      <c r="K10" s="23" t="n">
+      <c r="K10" s="24" t="n">
         <v>0.2149</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Webcam Pro</t>
@@ -1928,7 +1926,7 @@
       <c r="D11" s="17" t="n">
         <v>3170.67</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="25" t="n">
         <v>0.0473</v>
       </c>
       <c r="G11" s="16" t="inlineStr">
@@ -1945,26 +1943,26 @@
       <c r="J11" s="17" t="n">
         <v>152312.33</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="20" t="n">
         <v>0.1881</v>
       </c>
     </row>
     <row r="12" ht="8" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Bluetooth Headphones</t>
         </is>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B12" s="22" t="n">
         <v>655422.34</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <v>151</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="22" t="n">
         <v>2654.19</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="25" t="n">
         <v>0.053</v>
       </c>
     </row>
@@ -1986,28 +1984,28 @@
       <c r="E13" s="19" t="n">
         <v>0.0764</v>
       </c>
-      <c r="G13" s="24" t="inlineStr">
+      <c r="G13" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  MARKETING CAMPAIGN SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="20" t="inlineStr">
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>USB-C Hub</t>
         </is>
       </c>
-      <c r="B14" s="21" t="n">
+      <c r="B14" s="22" t="n">
         <v>506903.56</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="23" t="n">
         <v>161</v>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="22" t="n">
         <v>1911.33</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="19" t="n">
         <v>0.0683</v>
       </c>
       <c r="G14" s="15" t="inlineStr">
@@ -2036,7 +2034,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Laptop Stand</t>
@@ -2051,7 +2049,7 @@
       <c r="D15" s="17" t="n">
         <v>1307.75</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="25" t="n">
         <v>0.049</v>
       </c>
       <c r="G15" s="16" t="inlineStr">
@@ -2068,47 +2066,47 @@
       <c r="J15" s="17" t="n">
         <v>276020.3</v>
       </c>
-      <c r="K15" s="19" t="n">
+      <c r="K15" s="24" t="n">
         <v>0.2667</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Wireless Mouse</t>
         </is>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="22" t="n">
         <v>203728.2</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="23" t="n">
         <v>161</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="22" t="n">
         <v>798.97</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="24" t="n">
         <v>0.0373</v>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Organic</t>
         </is>
       </c>
-      <c r="H16" s="21" t="n">
+      <c r="H16" s="22" t="n">
         <v>946146.16</v>
       </c>
-      <c r="I16" s="22" t="n">
+      <c r="I16" s="23" t="n">
         <v>217</v>
       </c>
-      <c r="J16" s="21" t="n">
+      <c r="J16" s="22" t="n">
         <v>198461.91</v>
       </c>
-      <c r="K16" s="23" t="n">
+      <c r="K16" s="20" t="n">
         <v>0.2098</v>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="G17" s="16" t="inlineStr">
         <is>
           <t>Referral</t>
@@ -2123,35 +2121,35 @@
       <c r="J17" s="17" t="n">
         <v>185194.66</v>
       </c>
-      <c r="K17" s="19" t="n">
+      <c r="K17" s="20" t="n">
         <v>0.2048</v>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="25" t="inlineStr">
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">  PERFORMANCE BY REGION</t>
         </is>
       </c>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>Email Offer</t>
         </is>
       </c>
-      <c r="H18" s="21" t="n">
+      <c r="H18" s="22" t="n">
         <v>844455.76</v>
       </c>
-      <c r="I18" s="22" t="n">
+      <c r="I18" s="23" t="n">
         <v>222</v>
       </c>
-      <c r="J18" s="21" t="n">
+      <c r="J18" s="22" t="n">
         <v>117325.28</v>
       </c>
-      <c r="K18" s="23" t="n">
+      <c r="K18" s="19" t="n">
         <v>0.1389</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Region</t>
@@ -2191,11 +2189,11 @@
       <c r="J19" s="17" t="n">
         <v>158623.78</v>
       </c>
-      <c r="K19" s="19" t="n">
+      <c r="K19" s="20" t="n">
         <v>0.1959</v>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>West</t>
@@ -2210,47 +2208,47 @@
       <c r="D20" s="17" t="n">
         <v>273233.41</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="24" t="n">
         <v>0.0383</v>
       </c>
-      <c r="G20" s="20" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>Festive Sale</t>
         </is>
       </c>
-      <c r="H20" s="21" t="n">
+      <c r="H20" s="22" t="n">
         <v>789239.89</v>
       </c>
-      <c r="I20" s="22" t="n">
+      <c r="I20" s="23" t="n">
         <v>196</v>
       </c>
-      <c r="J20" s="21" t="n">
+      <c r="J20" s="22" t="n">
         <v>147123.38</v>
       </c>
-      <c r="K20" s="23" t="n">
+      <c r="K20" s="20" t="n">
         <v>0.1864</v>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="B21" s="21" t="n">
+      <c r="B21" s="22" t="n">
         <v>1301485.12</v>
       </c>
-      <c r="C21" s="22" t="n">
+      <c r="C21" s="23" t="n">
         <v>320</v>
       </c>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="22" t="n">
         <v>250426.93</v>
       </c>
-      <c r="E21" s="23" t="n">
+      <c r="E21" s="19" t="n">
         <v>0.07190000000000001</v>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="16" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>North</t>
@@ -2265,26 +2263,26 @@
       <c r="D22" s="17" t="n">
         <v>315503.55</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="25" t="n">
         <v>0.0569</v>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="B23" s="21" t="n">
+      <c r="B23" s="22" t="n">
         <v>1287643.6</v>
       </c>
-      <c r="C23" s="22" t="n">
+      <c r="C23" s="23" t="n">
         <v>292</v>
       </c>
-      <c r="D23" s="21" t="n">
+      <c r="D23" s="22" t="n">
         <v>243585.42</v>
       </c>
-      <c r="E23" s="23" t="n">
+      <c r="E23" s="24" t="n">
         <v>0.0411</v>
       </c>
     </row>
@@ -2320,6 +2318,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="005368A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2331,51 +2330,51 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
-        <is>
-          <t>MONTHLY SALES AND PROFIT TREND</t>
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>MONTHLY SALES AND PROFIT TREND  |  Jan 2025 – Mar 2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="5" customHeight="1"/>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="27" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
         <is>
           <t>Order Month</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B3" s="29" t="inlineStr">
         <is>
           <t>Total Revenue ($)</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="C3" s="29" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="29" t="inlineStr">
         <is>
           <t>Total Cost ($)</t>
         </is>
       </c>
-      <c r="E3" s="27" t="inlineStr">
+      <c r="E3" s="29" t="inlineStr">
         <is>
           <t>Gross Profit ($)</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="29" t="inlineStr">
         <is>
           <t>Profit Margin %</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
@@ -2392,34 +2391,34 @@
       <c r="E4" s="17" t="n">
         <v>78223.88</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="20" t="n">
         <v>0.1887</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="29" t="inlineStr">
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>2025-02</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="22" t="n">
         <v>381797.56</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="23" t="n">
         <v>84</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="22" t="n">
         <v>282834.36</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="22" t="n">
         <v>98963.2</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="24" t="n">
         <v>0.2592</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="28" t="inlineStr">
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>2025-03</t>
         </is>
@@ -2436,34 +2435,34 @@
       <c r="E6" s="17" t="n">
         <v>49121.5</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="20" t="n">
         <v>0.194</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="22" t="n">
         <v>361993.81</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>88</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="22" t="n">
         <v>299647.47</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="22" t="n">
         <v>62346.34</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.1722</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
@@ -2480,34 +2479,34 @@
       <c r="E8" s="17" t="n">
         <v>61825.89</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="20" t="n">
         <v>0.186</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="22" t="n">
         <v>373196.49</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <v>77</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="22" t="n">
         <v>305755.34</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="22" t="n">
         <v>67441.14999999999</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="32" t="n">
         <v>0.1807</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
@@ -2524,34 +2523,34 @@
       <c r="E10" s="17" t="n">
         <v>78689.63</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="20" t="n">
         <v>0.198</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>2025-08</t>
         </is>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="22" t="n">
         <v>334842.66</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="23" t="n">
         <v>94</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="22" t="n">
         <v>275722.86</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="22" t="n">
         <v>59119.8</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="32" t="n">
         <v>0.1766</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
@@ -2568,34 +2567,34 @@
       <c r="E12" s="17" t="n">
         <v>66536.2</v>
       </c>
-      <c r="F12" s="19" t="n">
+      <c r="F12" s="20" t="n">
         <v>0.1925</v>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="29" t="inlineStr">
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n">
+      <c r="B13" s="22" t="n">
         <v>364085.7</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <v>77</v>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="22" t="n">
         <v>292943.39</v>
       </c>
-      <c r="E13" s="21" t="n">
+      <c r="E13" s="22" t="n">
         <v>71142.31</v>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F13" s="32" t="n">
         <v>0.1954</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="28" t="inlineStr">
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>2025-11</t>
         </is>
@@ -2612,34 +2611,34 @@
       <c r="E14" s="17" t="n">
         <v>65449.77</v>
       </c>
-      <c r="F14" s="19" t="n">
+      <c r="F14" s="20" t="n">
         <v>0.1982</v>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15" s="22" t="n">
         <v>326024.85</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="23" t="n">
         <v>87</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="22" t="n">
         <v>264659.61</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="22" t="n">
         <v>61365.24</v>
       </c>
-      <c r="F15" s="23" t="n">
+      <c r="F15" s="32" t="n">
         <v>0.1882</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="28" t="inlineStr">
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
@@ -2656,34 +2655,34 @@
       <c r="E16" s="17" t="n">
         <v>134517.24</v>
       </c>
-      <c r="F16" s="19" t="n">
+      <c r="F16" s="24" t="n">
         <v>0.3044</v>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="22" t="n">
         <v>388410.22</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="23" t="n">
         <v>74</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="22" t="n">
         <v>317467.41</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="22" t="n">
         <v>70942.81</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="32" t="n">
         <v>0.1826</v>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="28" t="inlineStr">
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
@@ -2700,29 +2699,29 @@
       <c r="E18" s="17" t="n">
         <v>57064.35</v>
       </c>
-      <c r="F18" s="19" t="n">
+      <c r="F18" s="20" t="n">
         <v>0.2018</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n">
+      <c r="B19" s="34" t="n">
         <v>5328492.4</v>
       </c>
-      <c r="C19" s="32" t="n">
+      <c r="C19" s="35" t="n">
         <v>1250</v>
       </c>
-      <c r="D19" s="31" t="n">
+      <c r="D19" s="34" t="n">
         <v>4245778.09</v>
       </c>
-      <c r="E19" s="31" t="n">
+      <c r="E19" s="34" t="n">
         <v>1082548.82</v>
       </c>
-      <c r="F19" s="33" t="n">
+      <c r="F19" s="36" t="n">
         <v>0.2032</v>
       </c>
     </row>
@@ -2739,6 +2738,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C06000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2759,7 +2759,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>CATEGORY &amp; SEGMENT BREAKDOWNS</t>
         </is>
@@ -2772,13 +2772,13 @@
           <t xml:space="preserve">  SALES BY PRODUCT CATEGORY</t>
         </is>
       </c>
-      <c r="H3" s="24" t="inlineStr">
+      <c r="H3" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  SALES BY CUSTOMER SEGMENT</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Category</t>
@@ -2826,11 +2826,11 @@
       </c>
       <c r="K4" s="15" t="inlineStr">
         <is>
-          <t>Rev/Customer ($)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
+          <t>Rev / Customer ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Accessories</t>
@@ -2848,12 +2848,12 @@
       <c r="E5" s="17" t="n">
         <v>345746.17</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="20" t="n">
         <v>0.2148</v>
       </c>
-      <c r="H5" s="28" t="inlineStr">
-        <is>
-          <t>18-24</t>
+      <c r="H5" s="30" t="inlineStr">
+        <is>
+          <t>18–24</t>
         </is>
       </c>
       <c r="I5" s="17" t="n">
@@ -2866,43 +2866,43 @@
         <v>5746.53</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Wearables</t>
         </is>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="22" t="n">
         <v>1368209.84</v>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="23" t="n">
         <v>152</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="22" t="n">
         <v>6042.26</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="22" t="n">
         <v>208448.69</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.1524</v>
       </c>
-      <c r="H6" s="29" t="inlineStr">
-        <is>
-          <t>25-34</t>
-        </is>
-      </c>
-      <c r="I6" s="21" t="n">
+      <c r="H6" s="31" t="inlineStr">
+        <is>
+          <t>25–34</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="n">
         <v>1032052.93</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="23" t="n">
         <v>246</v>
       </c>
-      <c r="K6" s="21" t="n">
+      <c r="K6" s="22" t="n">
         <v>5639.63</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Audio</t>
@@ -2920,12 +2920,12 @@
       <c r="E7" s="17" t="n">
         <v>264390.68</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="20" t="n">
         <v>0.2106</v>
       </c>
-      <c r="H7" s="28" t="inlineStr">
-        <is>
-          <t>35-44</t>
+      <c r="H7" s="30" t="inlineStr">
+        <is>
+          <t>35–44</t>
         </is>
       </c>
       <c r="I7" s="17" t="n">
@@ -2934,48 +2934,48 @@
       <c r="J7" s="18" t="n">
         <v>268</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="K7" s="38" t="n">
         <v>6004.32</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n">
+      <c r="B8" s="22" t="n">
         <v>1094774.7</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>312</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="22" t="n">
         <v>2316.83</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="22" t="n">
         <v>264163.77</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="24" t="n">
         <v>0.2413</v>
       </c>
-      <c r="H8" s="29" t="inlineStr">
-        <is>
-          <t>45-54</t>
-        </is>
-      </c>
-      <c r="I8" s="21" t="n">
+      <c r="H8" s="31" t="inlineStr">
+        <is>
+          <t>45–54</t>
+        </is>
+      </c>
+      <c r="I8" s="22" t="n">
         <v>1059588.09</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="23" t="n">
         <v>267</v>
       </c>
-      <c r="K8" s="21" t="n">
+      <c r="K8" s="22" t="n">
         <v>5271.58</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="H9" s="28" t="inlineStr">
+    <row r="9" ht="16" customHeight="1">
+      <c r="H9" s="30" t="inlineStr">
         <is>
           <t>55+</t>
         </is>
@@ -2986,7 +2986,7 @@
       <c r="J9" s="18" t="n">
         <v>259</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="K9" s="38" t="n">
         <v>6222.92</v>
       </c>
     </row>

</xml_diff>